<commit_message>
Correct S28 perspective wording
</commit_message>
<xml_diff>
--- a/authoritative-materials/Creative_Leadership_Team_Profile_Question_Bank_V6_Final.xlsx
+++ b/authoritative-materials/Creative_Leadership_Team_Profile_Question_Bank_V6_Final.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R803abb1e4fe2482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rda9f533e636b4c7c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2614,7 +2614,7 @@
         <x:v>Section 3 - Team Dynamics for Effective Creation</x:v>
       </x:c>
       <x:c r="H47" s="10" t="str">
-        <x:v>...when we are under pressure to act quickly, it remains open to an intuitive insight that could change its current direction.</x:v>
+        <x:v>...when we are under pressure to act quickly, we remain open to an intuitive insight that could change our current direction.</x:v>
       </x:c>
       <x:c r="I47" s="10" t="str">
         <x:v>Almost never / Rarely/ About half the time / Often / Almost Always / No Opportunity to Observe</x:v>

</xml_diff>